<commit_message>
Pi power RC2: close source items - Waveshare data, Molex 43030-0038 + 18 AWG harness (16 AWG invalid), SSW-120-01-L-D, SMBJ15A row; budget re-run
PCB/interposer geometry unchanged; ERC/DRC/parity 0 on both projects.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ENatZXrEDA18PaxUrZWrpi
</commit_message>
<xml_diff>
--- a/OSBAMS_Pi_Display_Power_RevA_RC2/bom/OSBAMS_Pi_Display_Power_RevA_RC2_BOM.xlsx
+++ b/OSBAMS_Pi_Display_Power_RevA_RC2/bom/OSBAMS_Pi_Display_Power_RevA_RC2_BOM.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Footprint: official KiCad library (generated from manufacturer datasheet); NOT cross-checked against the manufacturer PDF</t>
+          <t>Electrical data USER-RELAYED from the Littelfuse SMBJ15A row (VRWM 15 V, VBR 16.7-18.5 V @ 1 mA, VC 24.4 V @ 24.6 A, IR 1 uA); footprint = KiCad library D_SMB (DO-214AA, cathode pad 1), not PDF-verified</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Mate: 43025-0200 + 43030 terminals</t>
+          <t>Mate: 43025-0200 + 43030-0038 terminals (18 AWG)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Mate: 43025-0400 + 43030 terminals</t>
+          <t>Mate: 43025-0400 + 43030-0038 terminals (18 AWG)</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Mate: 43025-0200 + 43030 terminals; same net as J_OUT (5V_PI / PI_GND, after F2)</t>
+          <t>Mate: 43025-0200 + 43030-0038 terminals (18 AWG); same net as J_OUT (5V_PI / PI_GND, after F2)</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Part number from the Molex family naming; mating-drawing not in project files</t>
+          <t>Mate of the 43045 header per Molex family naming; mating drawing not in project files</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Mates J_DISP 430450200 (keyed); display end connector per the Waveshare display data</t>
+          <t>Mates J_DISP 430450200 (keyed)</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>As above; display-end connector OPEN until the Waveshare data is available</t>
+          <t>As above; display end: MX1.25 2-pin per the Waveshare package cables (user-relayed) - confirm the housing</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Micro-Fit 3.0 female crimp terminals, 43030 family: 2 (J_IN) + 4 (J_OUT) + 2 (J_DISP) + 4 (interposer J1) = 12, correct size for the wire gauge used</t>
+          <t>Micro-Fit 3.0 female crimp terminals, 18 AWG / 0.75 mm2, tin: 2 (J_IN) + 4 (J_OUT) + 2 (J_DISP) + 4 (interposer J1) = 12 (+ spares)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>43030-xxxx - OWNER TO SELECT per wire gauge</t>
+          <t>43030-0038</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
@@ -1693,12 +1693,12 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Select from the Molex 43030 sales drawing: crimp range must cover 16 AWG (Pi branch) and the display/input wire; confirm current rating &gt;= 3 A per terminal</t>
+          <t>Crimp per Molex ATS-638280200: conductor crimp 1.00-1.10 mm, strip 2.54-2.92 mm, pull &gt;= 89 N; hand tool 63828-0200, locator 63828-0275; (-0039/-0040 = selective gold variants)</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>NOT VERIFIED - open harness item (does not affect the PCB)</t>
+          <t>VERIFIED for 18 AWG (Molex ATS-638280200, uploaded); no 16 AWG 43030 terminal exists; current rating with 18 AWG not in that file (first-article temperature check)</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       <c r="C30" s="2" t="inlineStr"/>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>16 AWG, &lt;=150 mm, 4 wires (Pi branch, red/black, 1:1 to the interposer); display feed 2 wires, gauge per display current</t>
+          <t>18 AWG UL1061-type, insulation OD &lt;= 1.85 mm, &lt;= 150 mm, 4 wires (Pi branch, red/black, 1:1 to the interposer); display feed 2 wires 18 AWG (or 20 AWG + 43030-0007), &lt;= 200 mm</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>owner to select</t>
+          <t>18 AWG UL1061-type (supplier by owner)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
@@ -1775,10 +1775,14 @@
           <t>Harness</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Insulation OD must be &lt;= 1.85 mm to fit the terminal insulation crimp</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>OPEN - harness item</t>
+          <t>Specified; supplier open</t>
         </is>
       </c>
     </row>

</xml_diff>